<commit_message>
Remove yellow/red cards and injuries (scoring, badges, pulls)
Cards: drop red_card/yellow_card from SCORING (index.html + daily_pull.py),
their scoring terms, stat columns, the admin stat-entry inputs, scoring-rules
table, stat sorts, breakdown rows and match-log tags. Also removes the
red-card suspension logic (suspendedNext) and its badge.

Injuries: remove injuries.json loading + the injury badge, delete
build_injuries.py, injuries.json and the injuries workflow. Photos/avatars
kept.

Source template regenerated without the card columns; tests updated (JS +
Python SCORING still asserted in sync). match_stats keeps its now-unused
card columns (harmless/additive).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UxX9exAz8Lj2F2Mhvw5TKH
</commit_message>
<xml_diff>
--- a/docs/rugby_scoring_source_template.xlsx
+++ b/docs/rugby_scoring_source_template.xlsx
@@ -353,25 +353,15 @@
     </comment>
     <comment ref="AF1" authorId="0" shapeId="0">
       <text>
-        <t>Red cards. -20 each.</t>
+        <t>Scrums won. Props +1.5, Hookers/Locks +1, Loose forwards +0.5, others 0.</t>
       </text>
     </comment>
     <comment ref="AG1" authorId="0" shapeId="0">
       <text>
-        <t>Yellow cards. -10 each.</t>
+        <t>Scrums lost. Props -3, Hookers/Locks -2, Loose forwards -1, others 0.</t>
       </text>
     </comment>
     <comment ref="AH1" authorId="0" shapeId="0">
-      <text>
-        <t>Scrums won. Props +1.5, Hookers/Locks +1, Loose forwards +0.5, others 0.</t>
-      </text>
-    </comment>
-    <comment ref="AI1" authorId="0" shapeId="0">
-      <text>
-        <t>Scrums lost. Props -3, Hookers/Locks -2, Loose forwards -1, others 0.</t>
-      </text>
-    </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0">
       <text>
         <t>Lineouts lost (own throw not secured). -2 each.</t>
       </text>
@@ -891,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ2"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -928,8 +918,6 @@
     <col width="15" customWidth="1" min="32" max="32"/>
     <col width="15" customWidth="1" min="33" max="33"/>
     <col width="15" customWidth="1" min="34" max="34"/>
-    <col width="15" customWidth="1" min="35" max="35"/>
-    <col width="15" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1090,25 +1078,15 @@
       </c>
       <c r="AF1" s="5" t="inlineStr">
         <is>
-          <t>red_cards</t>
+          <t>scrums_won</t>
         </is>
       </c>
       <c r="AG1" s="5" t="inlineStr">
         <is>
-          <t>yellow_cards</t>
+          <t>scrums_lost</t>
         </is>
       </c>
       <c r="AH1" s="5" t="inlineStr">
-        <is>
-          <t>scrums_won</t>
-        </is>
-      </c>
-      <c r="AI1" s="5" t="inlineStr">
-        <is>
-          <t>scrums_lost</t>
-        </is>
-      </c>
-      <c r="AJ1" s="5" t="inlineStr">
         <is>
           <t>lineouts_lost</t>
         </is>
@@ -1227,12 +1205,6 @@
         <v>0</v>
       </c>
       <c r="AH2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1368,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F440"/>
+  <dimension ref="A1:F481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6197,17 +6169,17 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Hooker</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -6229,17 +6201,17 @@
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -6261,12 +6233,12 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Hooker</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -6325,17 +6297,17 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Loose Forward</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -6485,17 +6457,17 @@
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Loose Forward</t>
         </is>
       </c>
       <c r="F160" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
@@ -6549,17 +6521,17 @@
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
         <is>
-          <t>Loose Forward</t>
+          <t>Hooker</t>
         </is>
       </c>
       <c r="F162" s="7" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -6741,17 +6713,17 @@
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>Loose Forward</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F168" s="7" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -6891,7 +6863,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Lucio Cintu</t>
+          <t>Lucio Cinti</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -6965,17 +6937,17 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -7157,17 +7129,17 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>FH</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Fly-half</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>HB</t>
         </is>
       </c>
     </row>
@@ -7285,17 +7257,17 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -7349,12 +7321,12 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Hooker</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -7413,12 +7385,12 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Hooker</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -7477,17 +7449,17 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Loose Forward</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -7509,12 +7481,12 @@
       </c>
       <c r="D192" s="7" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E192" s="7" t="inlineStr">
         <is>
-          <t>Hooker</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F192" s="7" t="inlineStr">
@@ -7605,17 +7577,17 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Loose Forward</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -7797,17 +7769,17 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Loose Forward</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
@@ -7829,17 +7801,17 @@
       </c>
       <c r="D202" s="7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="E202" s="7" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Loose Forward</t>
         </is>
       </c>
       <c r="F202" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
@@ -7957,17 +7929,17 @@
       </c>
       <c r="D206" s="7" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>SH</t>
         </is>
       </c>
       <c r="E206" s="7" t="inlineStr">
         <is>
-          <t>Outside Back</t>
+          <t>Scrum-half</t>
         </is>
       </c>
       <c r="F206" s="7" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>HB</t>
         </is>
       </c>
     </row>
@@ -7989,17 +7961,17 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>SH</t>
         </is>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Scrum-half</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>HB</t>
         </is>
       </c>
     </row>
@@ -8053,17 +8025,17 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>FH</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Fly-half</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>HB</t>
         </is>
       </c>
     </row>
@@ -8085,17 +8057,17 @@
       </c>
       <c r="D210" s="7" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="E210" s="7" t="inlineStr">
         <is>
-          <t>Outside Back</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F210" s="7" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>CE</t>
         </is>
       </c>
     </row>
@@ -8213,17 +8185,17 @@
       </c>
       <c r="D214" s="7" t="inlineStr">
         <is>
-          <t>SH</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E214" s="7" t="inlineStr">
         <is>
-          <t>Scrum-half</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F214" s="7" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -8245,17 +8217,17 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -8277,17 +8249,17 @@
       </c>
       <c r="D216" s="7" t="inlineStr">
         <is>
-          <t>FH</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E216" s="7" t="inlineStr">
         <is>
-          <t>Fly-half</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F216" s="7" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -8309,17 +8281,17 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -8341,17 +8313,17 @@
       </c>
       <c r="D218" s="7" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E218" s="7" t="inlineStr">
         <is>
-          <t>Hooker</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F218" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -8373,17 +8345,17 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>OB</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Outside Back</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>B3</t>
         </is>
       </c>
     </row>
@@ -8789,17 +8761,17 @@
       </c>
       <c r="D232" s="7" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E232" s="7" t="inlineStr">
         <is>
-          <t>Hooker</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F232" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -9813,17 +9785,17 @@
       </c>
       <c r="D264" s="7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="E264" s="7" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Loose Forward</t>
         </is>
       </c>
       <c r="F264" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
@@ -10325,17 +10297,17 @@
       </c>
       <c r="D280" s="7" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="E280" s="7" t="inlineStr">
         <is>
-          <t>Outside Back</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F280" s="7" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>CE</t>
         </is>
       </c>
     </row>
@@ -11189,17 +11161,17 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -11253,17 +11225,17 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Loose Forward</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -12149,17 +12121,17 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Loose Forward</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
@@ -12309,17 +12281,17 @@
       </c>
       <c r="D342" s="7" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="E342" s="7" t="inlineStr">
         <is>
-          <t>Outside Back</t>
+          <t>Hooker</t>
         </is>
       </c>
       <c r="F342" s="7" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -12501,17 +12473,17 @@
       </c>
       <c r="D348" s="7" t="inlineStr">
         <is>
-          <t>LK</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E348" s="7" t="inlineStr">
         <is>
-          <t>Lock</t>
+          <t>Prop</t>
         </is>
       </c>
       <c r="F348" s="7" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>FR</t>
         </is>
       </c>
     </row>
@@ -12693,17 +12665,17 @@
       </c>
       <c r="D354" s="7" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LK</t>
         </is>
       </c>
       <c r="E354" s="7" t="inlineStr">
         <is>
-          <t>Prop</t>
+          <t>Lock</t>
         </is>
       </c>
       <c r="F354" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>SR</t>
         </is>
       </c>
     </row>
@@ -13045,17 +13017,17 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>OB</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Outside Back</t>
+          <t>Centre</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>CE</t>
         </is>
       </c>
     </row>
@@ -15456,6 +15428,1318 @@
       <c r="F440" s="7" t="inlineStr">
         <is>
           <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>fra_33</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Reda Wardi</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="7" t="inlineStr">
+        <is>
+          <t>fra_34</t>
+        </is>
+      </c>
+      <c r="B442" s="7" t="inlineStr">
+        <is>
+          <t>Romain Ntamack</t>
+        </is>
+      </c>
+      <c r="C442" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D442" s="7" t="inlineStr">
+        <is>
+          <t>FH</t>
+        </is>
+      </c>
+      <c r="E442" s="7" t="inlineStr">
+        <is>
+          <t>Fly-half</t>
+        </is>
+      </c>
+      <c r="F442" s="7" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>fra_35</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Kalvin Gourgues</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="7" t="inlineStr">
+        <is>
+          <t>fra_36</t>
+        </is>
+      </c>
+      <c r="B444" s="7" t="inlineStr">
+        <is>
+          <t>Peato Mauvaka</t>
+        </is>
+      </c>
+      <c r="C444" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D444" s="7" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E444" s="7" t="inlineStr">
+        <is>
+          <t>Hooker</t>
+        </is>
+      </c>
+      <c r="F444" s="7" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>fra_37</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Emmanuel Meafou</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>LK</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="7" t="inlineStr">
+        <is>
+          <t>fra_38</t>
+        </is>
+      </c>
+      <c r="B446" s="7" t="inlineStr">
+        <is>
+          <t>Alexandre Roumat</t>
+        </is>
+      </c>
+      <c r="C446" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D446" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E446" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F446" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>fra_39</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Lenni Nouchi</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="7" t="inlineStr">
+        <is>
+          <t>fra_40</t>
+        </is>
+      </c>
+      <c r="B448" s="7" t="inlineStr">
+        <is>
+          <t>Auguste Cadot</t>
+        </is>
+      </c>
+      <c r="C448" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D448" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E448" s="7" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F448" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>fra_41</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Florien Verhaeghe</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>LK</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="7" t="inlineStr">
+        <is>
+          <t>rsa_47</t>
+        </is>
+      </c>
+      <c r="B450" s="7" t="inlineStr">
+        <is>
+          <t>Sacha Feinberg-Mngomezulu</t>
+        </is>
+      </c>
+      <c r="C450" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D450" s="7" t="inlineStr">
+        <is>
+          <t>FH</t>
+        </is>
+      </c>
+      <c r="E450" s="7" t="inlineStr">
+        <is>
+          <t>Fly-half</t>
+        </is>
+      </c>
+      <c r="F450" s="7" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>fra_42</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Antoine Dupont</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>SH</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Scrum-half</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="7" t="inlineStr">
+        <is>
+          <t>fra_43</t>
+        </is>
+      </c>
+      <c r="B452" s="7" t="inlineStr">
+        <is>
+          <t>Louis Bielle-Biarrey</t>
+        </is>
+      </c>
+      <c r="C452" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D452" s="7" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E452" s="7" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F452" s="7" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>rsa_48</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>RG Snyman</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>LK</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="7" t="inlineStr">
+        <is>
+          <t>rsa_49</t>
+        </is>
+      </c>
+      <c r="B454" s="7" t="inlineStr">
+        <is>
+          <t>Kwagga Smith</t>
+        </is>
+      </c>
+      <c r="C454" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D454" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E454" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F454" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>rsa_50</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Jean-Luc du Preez</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="7" t="inlineStr">
+        <is>
+          <t>rsa_51</t>
+        </is>
+      </c>
+      <c r="B456" s="7" t="inlineStr">
+        <is>
+          <t>Deon Fourie</t>
+        </is>
+      </c>
+      <c r="C456" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D456" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E456" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F456" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>rsa_52</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Juarno Augustus</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="7" t="inlineStr">
+        <is>
+          <t>rsa_53</t>
+        </is>
+      </c>
+      <c r="B458" s="7" t="inlineStr">
+        <is>
+          <t>Ruan Venter</t>
+        </is>
+      </c>
+      <c r="C458" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D458" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E458" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F458" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>rsa_54</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Jordan Hendrikse</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>FH</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Fly-half</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="7" t="inlineStr">
+        <is>
+          <t>rsa_55</t>
+        </is>
+      </c>
+      <c r="B460" s="7" t="inlineStr">
+        <is>
+          <t>Neethling Fouche</t>
+        </is>
+      </c>
+      <c r="C460" s="7" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D460" s="7" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="E460" s="7" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="F460" s="7" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>rsa_56</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Faf de Klerk</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>SH</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Scrum-half</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="7" t="inlineStr">
+        <is>
+          <t>eng_37</t>
+        </is>
+      </c>
+      <c r="B462" s="7" t="inlineStr">
+        <is>
+          <t>Maro Itoje</t>
+        </is>
+      </c>
+      <c r="C462" s="7" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D462" s="7" t="inlineStr">
+        <is>
+          <t>LK</t>
+        </is>
+      </c>
+      <c r="E462" s="7" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="F462" s="7" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>eng_38</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Sam Underhill</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="7" t="inlineStr">
+        <is>
+          <t>fra_44</t>
+        </is>
+      </c>
+      <c r="B464" s="7" t="inlineStr">
+        <is>
+          <t>Thomas Ramos</t>
+        </is>
+      </c>
+      <c r="C464" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D464" s="7" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E464" s="7" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F464" s="7" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>fra_45</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Gael Fickou</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="7" t="inlineStr">
+        <is>
+          <t>fra_46</t>
+        </is>
+      </c>
+      <c r="B466" s="7" t="inlineStr">
+        <is>
+          <t>Charles Ollivon</t>
+        </is>
+      </c>
+      <c r="C466" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D466" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E466" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F466" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>ire_37</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Mack Hansen</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="7" t="inlineStr">
+        <is>
+          <t>nzl_35</t>
+        </is>
+      </c>
+      <c r="B468" s="7" t="inlineStr">
+        <is>
+          <t>Ethan Blackadder</t>
+        </is>
+      </c>
+      <c r="C468" s="7" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D468" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E468" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F468" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>aus_38</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Darby Lancaster</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="7" t="inlineStr">
+        <is>
+          <t>sco_37</t>
+        </is>
+      </c>
+      <c r="B470" s="7" t="inlineStr">
+        <is>
+          <t>Matt Currie</t>
+        </is>
+      </c>
+      <c r="C470" s="7" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
+      <c r="D470" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E470" s="7" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F470" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>ita_34</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Ange Capuozzo</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="7" t="inlineStr">
+        <is>
+          <t>ita_35</t>
+        </is>
+      </c>
+      <c r="B472" s="7" t="inlineStr">
+        <is>
+          <t>Sebasitan Negri</t>
+        </is>
+      </c>
+      <c r="C472" s="7" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D472" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E472" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F472" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>ita_36</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Simone Ferrari</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="7" t="inlineStr">
+        <is>
+          <t>ita_37</t>
+        </is>
+      </c>
+      <c r="B474" s="7" t="inlineStr">
+        <is>
+          <t>Manuel Zuliani</t>
+        </is>
+      </c>
+      <c r="C474" s="7" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D474" s="7" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E474" s="7" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F474" s="7" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>ita_38</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Jacopo Trulla</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="7" t="inlineStr">
+        <is>
+          <t>fij_33</t>
+        </is>
+      </c>
+      <c r="B476" s="7" t="inlineStr">
+        <is>
+          <t>Iosefo Masi</t>
+        </is>
+      </c>
+      <c r="C476" s="7" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="D476" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E476" s="7" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F476" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>arg_35</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Facundo Isa</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="7" t="inlineStr">
+        <is>
+          <t>arg_36</t>
+        </is>
+      </c>
+      <c r="B478" s="7" t="inlineStr">
+        <is>
+          <t>Jeronimo De La Fuente</t>
+        </is>
+      </c>
+      <c r="C478" s="7" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D478" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E478" s="7" t="inlineStr">
+        <is>
+          <t>Centre</t>
+        </is>
+      </c>
+      <c r="F478" s="7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>fra_47</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Francois Cros</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="7" t="inlineStr">
+        <is>
+          <t>fra_48</t>
+        </is>
+      </c>
+      <c r="B480" s="7" t="inlineStr">
+        <is>
+          <t>Thibaud Flament</t>
+        </is>
+      </c>
+      <c r="C480" s="7" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D480" s="7" t="inlineStr">
+        <is>
+          <t>LK</t>
+        </is>
+      </c>
+      <c r="E480" s="7" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="F480" s="7" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>fra_49</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Anthony Jelonch</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>LF</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Loose Forward</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>BR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore card scoring (badge stays removed) + squad update 6
Cards: the previous change removed yellow/red cards entirely; per feedback,
restore the SCORING (index.html + daily_pull.py), stat columns, admin inputs,
scoring-rules table, stat sorts, breakdown and match-log tags, and the
template columns. Only the card-derived suspension BADGE (and injuries) stay
removed. JS/Python SCORING re-asserted in sync.

Squad update: +2 players (Livai Natave, Sam Greene), 0 removed, all ids and
positions unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UxX9exAz8Lj2F2Mhvw5TKH
</commit_message>
<xml_diff>
--- a/docs/rugby_scoring_source_template.xlsx
+++ b/docs/rugby_scoring_source_template.xlsx
@@ -353,15 +353,25 @@
     </comment>
     <comment ref="AF1" authorId="0" shapeId="0">
       <text>
-        <t>Scrums won. Props +1.5, Hookers/Locks +1, Loose forwards +0.5, others 0.</t>
+        <t>Red cards. -20 each.</t>
       </text>
     </comment>
     <comment ref="AG1" authorId="0" shapeId="0">
       <text>
+        <t>Yellow cards. -10 each.</t>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0" shapeId="0">
+      <text>
+        <t>Scrums won. Props +1.5, Hookers/Locks +1, Loose forwards +0.5, others 0.</t>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="0" shapeId="0">
+      <text>
         <t>Scrums lost. Props -3, Hookers/Locks -2, Loose forwards -1, others 0.</t>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
+    <comment ref="AJ1" authorId="0" shapeId="0">
       <text>
         <t>Lineouts lost (own throw not secured). -2 each.</t>
       </text>
@@ -881,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AJ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -918,6 +928,8 @@
     <col width="15" customWidth="1" min="32" max="32"/>
     <col width="15" customWidth="1" min="33" max="33"/>
     <col width="15" customWidth="1" min="34" max="34"/>
+    <col width="15" customWidth="1" min="35" max="35"/>
+    <col width="15" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1078,15 +1090,25 @@
       </c>
       <c r="AF1" s="5" t="inlineStr">
         <is>
+          <t>red_cards</t>
+        </is>
+      </c>
+      <c r="AG1" s="5" t="inlineStr">
+        <is>
+          <t>yellow_cards</t>
+        </is>
+      </c>
+      <c r="AH1" s="5" t="inlineStr">
+        <is>
           <t>scrums_won</t>
         </is>
       </c>
-      <c r="AG1" s="5" t="inlineStr">
+      <c r="AI1" s="5" t="inlineStr">
         <is>
           <t>scrums_lost</t>
         </is>
       </c>
-      <c r="AH1" s="5" t="inlineStr">
+      <c r="AJ1" s="5" t="inlineStr">
         <is>
           <t>lineouts_lost</t>
         </is>
@@ -1205,6 +1227,12 @@
         <v>0</v>
       </c>
       <c r="AH2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1340,7 +1368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F481"/>
+  <dimension ref="A1:F483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16740,6 +16768,70 @@
       <c r="F481" t="inlineStr">
         <is>
           <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="7" t="inlineStr">
+        <is>
+          <t>fij_34</t>
+        </is>
+      </c>
+      <c r="B482" s="7" t="inlineStr">
+        <is>
+          <t>Livai Natave</t>
+        </is>
+      </c>
+      <c r="C482" s="7" t="inlineStr">
+        <is>
+          <t>Fiji</t>
+        </is>
+      </c>
+      <c r="D482" s="7" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="E482" s="7" t="inlineStr">
+        <is>
+          <t>Prop</t>
+        </is>
+      </c>
+      <c r="F482" s="7" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>jpn_36</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Sam Greene</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Outside Back</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>B3</t>
         </is>
       </c>
     </row>

</xml_diff>